<commit_message>
manejo de formato monetario en columnas adicionales
</commit_message>
<xml_diff>
--- a/shared/Comisiones_2026_10.xlsx
+++ b/shared/Comisiones_2026_10.xlsx
@@ -928,7 +928,7 @@
     <x:col min="6" max="6" width="7.853482" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="9.424911" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="7.853482" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10.424911" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.996339" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="9.424911" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="3.996339" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="4.996339" style="0" customWidth="1"/>
@@ -1028,7 +1028,7 @@
       <x:c r="H6" s="6">
         <x:v>17.26</x:v>
       </x:c>
-      <x:c r="I6" s="6">
+      <x:c r="I6" s="5">
         <x:v>46268.5951388889</x:v>
       </x:c>
       <x:c r="J6" s="6">
@@ -1069,7 +1069,7 @@
       <x:c r="H7" s="6">
         <x:v>38.72</x:v>
       </x:c>
-      <x:c r="I7" s="6">
+      <x:c r="I7" s="5">
         <x:v>46269.4923611111</x:v>
       </x:c>
       <x:c r="J7" s="6">
@@ -1110,7 +1110,7 @@
       <x:c r="H8" s="6">
         <x:v>17.5</x:v>
       </x:c>
-      <x:c r="I8" s="6">
+      <x:c r="I8" s="5">
         <x:v>46269.4951388889</x:v>
       </x:c>
       <x:c r="J8" s="6">
@@ -1151,7 +1151,7 @@
       <x:c r="H9" s="6">
         <x:v>21.04</x:v>
       </x:c>
-      <x:c r="I9" s="6">
+      <x:c r="I9" s="5">
         <x:v>46269.4951388889</x:v>
       </x:c>
       <x:c r="J9" s="6">
@@ -1192,7 +1192,7 @@
       <x:c r="H10" s="6">
         <x:v>10.4</x:v>
       </x:c>
-      <x:c r="I10" s="6">
+      <x:c r="I10" s="5">
         <x:v>46269.4951388889</x:v>
       </x:c>
       <x:c r="J10" s="6">
@@ -1233,7 +1233,7 @@
       <x:c r="H11" s="6">
         <x:v>33.95</x:v>
       </x:c>
-      <x:c r="I11" s="6">
+      <x:c r="I11" s="5">
         <x:v>46272.3736111111</x:v>
       </x:c>
       <x:c r="J11" s="6">
@@ -1274,7 +1274,7 @@
       <x:c r="H12" s="6">
         <x:v>2.74</x:v>
       </x:c>
-      <x:c r="I12" s="6">
+      <x:c r="I12" s="5">
         <x:v>46272.375</x:v>
       </x:c>
       <x:c r="J12" s="6">
@@ -1315,7 +1315,7 @@
       <x:c r="H13" s="6">
         <x:v>6.11</x:v>
       </x:c>
-      <x:c r="I13" s="6">
+      <x:c r="I13" s="5">
         <x:v>46272.3805555556</x:v>
       </x:c>
       <x:c r="J13" s="6">
@@ -1356,7 +1356,7 @@
       <x:c r="H14" s="6">
         <x:v>28.51</x:v>
       </x:c>
-      <x:c r="I14" s="6">
+      <x:c r="I14" s="5">
         <x:v>46272.3826388889</x:v>
       </x:c>
       <x:c r="J14" s="6">
@@ -1397,7 +1397,7 @@
       <x:c r="H15" s="6">
         <x:v>68.13</x:v>
       </x:c>
-      <x:c r="I15" s="6">
+      <x:c r="I15" s="5">
         <x:v>46272.3951388889</x:v>
       </x:c>
       <x:c r="J15" s="6">
@@ -1438,7 +1438,7 @@
       <x:c r="H16" s="6">
         <x:v>15.61</x:v>
       </x:c>
-      <x:c r="I16" s="6">
+      <x:c r="I16" s="5">
         <x:v>46272.5875</x:v>
       </x:c>
       <x:c r="J16" s="6">
@@ -1479,7 +1479,7 @@
       <x:c r="H17" s="6">
         <x:v>11.02</x:v>
       </x:c>
-      <x:c r="I17" s="6">
+      <x:c r="I17" s="5">
         <x:v>46272.5875</x:v>
       </x:c>
       <x:c r="J17" s="6">
@@ -1520,7 +1520,7 @@
       <x:c r="H18" s="6">
         <x:v>47.63</x:v>
       </x:c>
-      <x:c r="I18" s="6">
+      <x:c r="I18" s="5">
         <x:v>46272.5895833333</x:v>
       </x:c>
       <x:c r="J18" s="6">
@@ -1561,7 +1561,7 @@
       <x:c r="H19" s="6">
         <x:v>85.32</x:v>
       </x:c>
-      <x:c r="I19" s="6">
+      <x:c r="I19" s="5">
         <x:v>46275.4833333333</x:v>
       </x:c>
       <x:c r="J19" s="6">
@@ -1602,7 +1602,7 @@
       <x:c r="H20" s="6">
         <x:v>476.34</x:v>
       </x:c>
-      <x:c r="I20" s="6">
+      <x:c r="I20" s="5">
         <x:v>46275.4833333333</x:v>
       </x:c>
       <x:c r="J20" s="6">
@@ -1643,7 +1643,7 @@
       <x:c r="H21" s="6">
         <x:v>19.69</x:v>
       </x:c>
-      <x:c r="I21" s="6">
+      <x:c r="I21" s="5">
         <x:v>46276.4486111111</x:v>
       </x:c>
       <x:c r="J21" s="6">
@@ -1684,7 +1684,7 @@
       <x:c r="H22" s="6">
         <x:v>36.75</x:v>
       </x:c>
-      <x:c r="I22" s="6">
+      <x:c r="I22" s="5">
         <x:v>46276.4618055556</x:v>
       </x:c>
       <x:c r="J22" s="6">
@@ -1725,7 +1725,7 @@
       <x:c r="H23" s="6">
         <x:v>2.6</x:v>
       </x:c>
-      <x:c r="I23" s="6">
+      <x:c r="I23" s="5">
         <x:v>46276.4618055556</x:v>
       </x:c>
       <x:c r="J23" s="6">
@@ -1766,7 +1766,7 @@
       <x:c r="H24" s="6">
         <x:v>35.57</x:v>
       </x:c>
-      <x:c r="I24" s="6">
+      <x:c r="I24" s="5">
         <x:v>46276.6</x:v>
       </x:c>
       <x:c r="J24" s="6">
@@ -1807,7 +1807,7 @@
       <x:c r="H25" s="6">
         <x:v>55.34</x:v>
       </x:c>
-      <x:c r="I25" s="6">
+      <x:c r="I25" s="5">
         <x:v>46276.6</x:v>
       </x:c>
       <x:c r="J25" s="6">
@@ -1848,7 +1848,7 @@
       <x:c r="H26" s="6">
         <x:v>48.64</x:v>
       </x:c>
-      <x:c r="I26" s="6">
+      <x:c r="I26" s="5">
         <x:v>46276.6027777778</x:v>
       </x:c>
       <x:c r="J26" s="6">
@@ -1889,7 +1889,7 @@
       <x:c r="H27" s="6">
         <x:v>20.82</x:v>
       </x:c>
-      <x:c r="I27" s="6">
+      <x:c r="I27" s="5">
         <x:v>46279.6041666667</x:v>
       </x:c>
       <x:c r="J27" s="6">
@@ -1930,7 +1930,7 @@
       <x:c r="H28" s="6">
         <x:v>140.52</x:v>
       </x:c>
-      <x:c r="I28" s="6">
+      <x:c r="I28" s="5">
         <x:v>46280.4722222222</x:v>
       </x:c>
       <x:c r="J28" s="6">
@@ -1971,7 +1971,7 @@
       <x:c r="H29" s="6">
         <x:v>48.79</x:v>
       </x:c>
-      <x:c r="I29" s="6">
+      <x:c r="I29" s="5">
         <x:v>46280.6833333333</x:v>
       </x:c>
       <x:c r="J29" s="6">
@@ -2012,7 +2012,7 @@
       <x:c r="H30" s="6">
         <x:v>20.81</x:v>
       </x:c>
-      <x:c r="I30" s="6">
+      <x:c r="I30" s="5">
         <x:v>46281.4805555556</x:v>
       </x:c>
       <x:c r="J30" s="6">
@@ -2053,7 +2053,7 @@
       <x:c r="H31" s="6">
         <x:v>193.93</x:v>
       </x:c>
-      <x:c r="I31" s="6">
+      <x:c r="I31" s="5">
         <x:v>46281.4819444444</x:v>
       </x:c>
       <x:c r="J31" s="6">
@@ -2094,7 +2094,7 @@
       <x:c r="H32" s="6">
         <x:v>73.44</x:v>
       </x:c>
-      <x:c r="I32" s="6">
+      <x:c r="I32" s="5">
         <x:v>46281.4826388889</x:v>
       </x:c>
       <x:c r="J32" s="6">
@@ -2135,7 +2135,7 @@
       <x:c r="H33" s="6">
         <x:v>210.14</x:v>
       </x:c>
-      <x:c r="I33" s="6">
+      <x:c r="I33" s="5">
         <x:v>46281.4840277778</x:v>
       </x:c>
       <x:c r="J33" s="6">
@@ -2176,7 +2176,7 @@
       <x:c r="H34" s="6">
         <x:v>77.52</x:v>
       </x:c>
-      <x:c r="I34" s="6">
+      <x:c r="I34" s="5">
         <x:v>46281.4854166667</x:v>
       </x:c>
       <x:c r="J34" s="6">
@@ -2217,7 +2217,7 @@
       <x:c r="H35" s="6">
         <x:v>21.82</x:v>
       </x:c>
-      <x:c r="I35" s="6">
+      <x:c r="I35" s="5">
         <x:v>46281.4868055556</x:v>
       </x:c>
       <x:c r="J35" s="6">
@@ -2258,7 +2258,7 @@
       <x:c r="H36" s="6">
         <x:v>23.9</x:v>
       </x:c>
-      <x:c r="I36" s="6">
+      <x:c r="I36" s="5">
         <x:v>46281.4895833333</x:v>
       </x:c>
       <x:c r="J36" s="6">
@@ -2299,7 +2299,7 @@
       <x:c r="H37" s="6">
         <x:v>212.91</x:v>
       </x:c>
-      <x:c r="I37" s="6">
+      <x:c r="I37" s="5">
         <x:v>46282.3666666667</x:v>
       </x:c>
       <x:c r="J37" s="6">
@@ -2340,7 +2340,7 @@
       <x:c r="H38" s="6">
         <x:v>36.19</x:v>
       </x:c>
-      <x:c r="I38" s="6">
+      <x:c r="I38" s="5">
         <x:v>46282.3854166667</x:v>
       </x:c>
       <x:c r="J38" s="6">
@@ -2381,7 +2381,7 @@
       <x:c r="H39" s="6">
         <x:v>36.43</x:v>
       </x:c>
-      <x:c r="I39" s="6">
+      <x:c r="I39" s="5">
         <x:v>46282.4381944444</x:v>
       </x:c>
       <x:c r="J39" s="6">
@@ -2422,7 +2422,7 @@
       <x:c r="H40" s="6">
         <x:v>55.08</x:v>
       </x:c>
-      <x:c r="I40" s="6">
+      <x:c r="I40" s="5">
         <x:v>46283.6111111111</x:v>
       </x:c>
       <x:c r="J40" s="6">
@@ -2463,7 +2463,7 @@
       <x:c r="H41" s="6">
         <x:v>22.02</x:v>
       </x:c>
-      <x:c r="I41" s="6">
+      <x:c r="I41" s="5">
         <x:v>46283.6131944444</x:v>
       </x:c>
       <x:c r="J41" s="6">
@@ -2504,7 +2504,7 @@
       <x:c r="H42" s="6">
         <x:v>94.94</x:v>
       </x:c>
-      <x:c r="I42" s="6">
+      <x:c r="I42" s="5">
         <x:v>46283.6152777778</x:v>
       </x:c>
       <x:c r="J42" s="6">
@@ -2545,7 +2545,7 @@
       <x:c r="H43" s="6">
         <x:v>503.79</x:v>
       </x:c>
-      <x:c r="I43" s="6">
+      <x:c r="I43" s="5">
         <x:v>46283.6986111111</x:v>
       </x:c>
       <x:c r="J43" s="6">
@@ -2586,7 +2586,7 @@
       <x:c r="H44" s="6">
         <x:v>10.65</x:v>
       </x:c>
-      <x:c r="I44" s="6">
+      <x:c r="I44" s="5">
         <x:v>46286.4090277778</x:v>
       </x:c>
       <x:c r="J44" s="6">
@@ -2627,7 +2627,7 @@
       <x:c r="H45" s="6">
         <x:v>27.41</x:v>
       </x:c>
-      <x:c r="I45" s="6">
+      <x:c r="I45" s="5">
         <x:v>46286.6048611111</x:v>
       </x:c>
       <x:c r="J45" s="6">
@@ -2668,7 +2668,7 @@
       <x:c r="H46" s="6">
         <x:v>28.37</x:v>
       </x:c>
-      <x:c r="I46" s="6">
+      <x:c r="I46" s="5">
         <x:v>46286.6451388889</x:v>
       </x:c>
       <x:c r="J46" s="6">
@@ -2709,7 +2709,7 @@
       <x:c r="H47" s="6">
         <x:v>35.56</x:v>
       </x:c>
-      <x:c r="I47" s="6">
+      <x:c r="I47" s="5">
         <x:v>46286.6451388889</x:v>
       </x:c>
       <x:c r="J47" s="6">
@@ -2750,7 +2750,7 @@
       <x:c r="H48" s="6">
         <x:v>60.05</x:v>
       </x:c>
-      <x:c r="I48" s="6">
+      <x:c r="I48" s="5">
         <x:v>46287.45</x:v>
       </x:c>
       <x:c r="J48" s="6">
@@ -2791,7 +2791,7 @@
       <x:c r="H49" s="6">
         <x:v>58.28</x:v>
       </x:c>
-      <x:c r="I49" s="6">
+      <x:c r="I49" s="5">
         <x:v>46287.45</x:v>
       </x:c>
       <x:c r="J49" s="6">
@@ -2832,7 +2832,7 @@
       <x:c r="H50" s="6">
         <x:v>85.78</x:v>
       </x:c>
-      <x:c r="I50" s="6">
+      <x:c r="I50" s="5">
         <x:v>46288.6305555556</x:v>
       </x:c>
       <x:c r="J50" s="6">
@@ -2873,7 +2873,7 @@
       <x:c r="H51" s="6">
         <x:v>60.89</x:v>
       </x:c>
-      <x:c r="I51" s="6">
+      <x:c r="I51" s="5">
         <x:v>46290.3486111111</x:v>
       </x:c>
       <x:c r="J51" s="6">
@@ -2914,7 +2914,7 @@
       <x:c r="H52" s="6">
         <x:v>18.51</x:v>
       </x:c>
-      <x:c r="I52" s="6">
+      <x:c r="I52" s="5">
         <x:v>46290.4430555556</x:v>
       </x:c>
       <x:c r="J52" s="6">
@@ -2955,7 +2955,7 @@
       <x:c r="H53" s="6">
         <x:v>153.77</x:v>
       </x:c>
-      <x:c r="I53" s="6">
+      <x:c r="I53" s="5">
         <x:v>46293.4513888889</x:v>
       </x:c>
       <x:c r="J53" s="6">
@@ -2996,7 +2996,7 @@
       <x:c r="H54" s="6">
         <x:v>58.81</x:v>
       </x:c>
-      <x:c r="I54" s="6">
+      <x:c r="I54" s="5">
         <x:v>46294.3993055556</x:v>
       </x:c>
       <x:c r="J54" s="6">
@@ -3037,7 +3037,7 @@
       <x:c r="H55" s="6">
         <x:v>15.15</x:v>
       </x:c>
-      <x:c r="I55" s="6">
+      <x:c r="I55" s="5">
         <x:v>46294.4020833333</x:v>
       </x:c>
       <x:c r="J55" s="6">
@@ -3078,7 +3078,7 @@
       <x:c r="H56" s="6">
         <x:v>13.13</x:v>
       </x:c>
-      <x:c r="I56" s="6">
+      <x:c r="I56" s="5">
         <x:v>46294.5909722222</x:v>
       </x:c>
       <x:c r="J56" s="6">
@@ -3251,7 +3251,7 @@
       <x:c r="H6" s="6">
         <x:v>229.69</x:v>
       </x:c>
-      <x:c r="I6" s="6">
+      <x:c r="I6" s="5">
         <x:v>46272.3798611111</x:v>
       </x:c>
       <x:c r="J6" s="6">
@@ -3292,7 +3292,7 @@
       <x:c r="H7" s="6">
         <x:v>12.29</x:v>
       </x:c>
-      <x:c r="I7" s="6">
+      <x:c r="I7" s="5">
         <x:v>46290.4895833333</x:v>
       </x:c>
       <x:c r="J7" s="6">
@@ -3367,7 +3367,7 @@
     <x:col min="6" max="6" width="9.853482" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="9.424911" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="7.853482" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10.424911" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.996339" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="17.424911" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="3.996339" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="4.996339" style="0" customWidth="1"/>
@@ -3467,7 +3467,7 @@
       <x:c r="H6" s="6">
         <x:v>63.13</x:v>
       </x:c>
-      <x:c r="I6" s="6">
+      <x:c r="I6" s="5">
         <x:v>46268.4770833333</x:v>
       </x:c>
       <x:c r="J6" s="6">
@@ -3508,7 +3508,7 @@
       <x:c r="H7" s="6">
         <x:v>43.72</x:v>
       </x:c>
-      <x:c r="I7" s="6">
+      <x:c r="I7" s="5">
         <x:v>46272.3965277778</x:v>
       </x:c>
       <x:c r="J7" s="6">
@@ -3549,7 +3549,7 @@
       <x:c r="H8" s="6">
         <x:v>16.66</x:v>
       </x:c>
-      <x:c r="I8" s="6">
+      <x:c r="I8" s="5">
         <x:v>46281.4902777778</x:v>
       </x:c>
       <x:c r="J8" s="6">
@@ -3590,7 +3590,7 @@
       <x:c r="H9" s="6">
         <x:v>60.34</x:v>
       </x:c>
-      <x:c r="I9" s="6">
+      <x:c r="I9" s="5">
         <x:v>46283.6722222222</x:v>
       </x:c>
       <x:c r="J9" s="6">
@@ -3631,7 +3631,7 @@
       <x:c r="H10" s="6">
         <x:v>118.28</x:v>
       </x:c>
-      <x:c r="I10" s="6">
+      <x:c r="I10" s="5">
         <x:v>46283.6736111111</x:v>
       </x:c>
       <x:c r="J10" s="6">
@@ -3672,7 +3672,7 @@
       <x:c r="H11" s="6">
         <x:v>33.59</x:v>
       </x:c>
-      <x:c r="I11" s="6">
+      <x:c r="I11" s="5">
         <x:v>46283.6770833333</x:v>
       </x:c>
       <x:c r="J11" s="6">
@@ -3713,7 +3713,7 @@
       <x:c r="H12" s="6">
         <x:v>28.07</x:v>
       </x:c>
-      <x:c r="I12" s="6">
+      <x:c r="I12" s="5">
         <x:v>46283.6833333333</x:v>
       </x:c>
       <x:c r="J12" s="6">
@@ -3754,7 +3754,7 @@
       <x:c r="H13" s="6">
         <x:v>498.07</x:v>
       </x:c>
-      <x:c r="I13" s="6">
+      <x:c r="I13" s="5">
         <x:v>46293.4826388889</x:v>
       </x:c>
       <x:c r="J13" s="6">
@@ -3795,7 +3795,7 @@
       <x:c r="H14" s="6">
         <x:v>110.94</x:v>
       </x:c>
-      <x:c r="I14" s="6">
+      <x:c r="I14" s="5">
         <x:v>46294.6076388889</x:v>
       </x:c>
       <x:c r="J14" s="6">
@@ -3868,7 +3868,7 @@
     <x:col min="4" max="4" width="8.996339" style="0" customWidth="1"/>
     <x:col min="5" max="7" width="7.853482" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="6.567768" style="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10.424911" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.996339" style="0" customWidth="1"/>
     <x:col min="10" max="10" width="17.424911" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="2.996339" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="4.996339" style="0" customWidth="1"/>
@@ -3968,7 +3968,7 @@
       <x:c r="H6" s="6">
         <x:v>188.68</x:v>
       </x:c>
-      <x:c r="I6" s="6">
+      <x:c r="I6" s="5">
         <x:v>46296.3756944444</x:v>
       </x:c>
       <x:c r="J6" s="6">
@@ -4009,7 +4009,7 @@
       <x:c r="H7" s="6">
         <x:v>51.79</x:v>
       </x:c>
-      <x:c r="I7" s="6">
+      <x:c r="I7" s="5">
         <x:v>46296.5680555556</x:v>
       </x:c>
       <x:c r="J7" s="6">
@@ -4050,7 +4050,7 @@
       <x:c r="H8" s="6">
         <x:v>22.3</x:v>
       </x:c>
-      <x:c r="I8" s="6">
+      <x:c r="I8" s="5">
         <x:v>46296.5680555556</x:v>
       </x:c>
       <x:c r="J8" s="6">
@@ -4224,7 +4224,7 @@
       <x:c r="H6" s="6">
         <x:v>497.37</x:v>
       </x:c>
-      <x:c r="I6" s="6">
+      <x:c r="I6" s="5">
         <x:v>46296.3770833333</x:v>
       </x:c>
       <x:c r="J6" s="6">
@@ -4265,7 +4265,7 @@
       <x:c r="H7" s="6">
         <x:v>243</x:v>
       </x:c>
-      <x:c r="I7" s="6">
+      <x:c r="I7" s="5">
         <x:v>46296.3965277778</x:v>
       </x:c>
       <x:c r="J7" s="6">

</xml_diff>